<commit_message>
Initial saving of dxf for pivot tables
The style part saving code originally saved all registered dxf, not
only used. That didn't crash, but saved unused dxfs.

The code now only saves used dxfs. Used dxfs are then saved to styles
part and registered to SaveContext (previously even unused dxfs were
saved). Workbook shouldn't save unused parts (e.g. intermediate state
of dxf that was being changed is still registered, even if it isn't
used). The bad things is that other tests that use dxf started to fail,
because they are trying to find dxfId in SaveContext, but it is no
longer there. Will be fixed later.

The dxf saving code was updated due to new dxf store structure.

The XLPivotFieldStyleFormatsTests test files are essentially only
updated to new XML format without all the clutter like namespaces and
default values. Validated through XML compare and visually.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/PivotTable/Style/Modify_pivot_field_label_style.xlsx
+++ b/ClosedXML.Tests/Resource/Other/PivotTable/Style/Modify_pivot_field_label_style.xlsx
@@ -44,75 +44,64 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-  <x:dxfs count="1">
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:strike/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:fgColor auto="1"/>
-          <x:bgColor rgb="FFD3D3D3"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-  </x:dxfs>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b/>
+        <strike/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD3D3D3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/pivotTables/pivotTable.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>